<commit_message>
Update recipient data in Excel file
</commit_message>
<xml_diff>
--- a/UseCase__002_.xlsx
+++ b/UseCase__002_.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Music\Notifier\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2575749F-D50D-496D-9E84-6CC488CD7E66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52EF912D-C04B-488D-AB5F-BF9682BB42B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="2" xr2:uid="{64A6A2CA-9133-4B66-AF2E-02D028F69B9C}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{64A6A2CA-9133-4B66-AF2E-02D028F69B9C}"/>
   </bookViews>
   <sheets>
     <sheet name="ProdUser" sheetId="1" r:id="rId1"/>
@@ -80,16 +80,16 @@
     <t>abcd1234@gmail.com</t>
   </si>
   <si>
-    <t>manibhushan47071@gmail.com</t>
-  </si>
-  <si>
-    <t>chhoti06112002@gmail.com</t>
-  </si>
-  <si>
     <t>defg789@gmail</t>
   </si>
   <si>
     <t>&lt;body&gt;  &lt;p&gt;  &lt;font face="Arial" size="2"&gt;Hello [Name], &lt;/font&gt;  &lt;/p&gt;  &lt;p&gt;  &lt;font face="Arial" size="2"&gt;&lt;/font&gt;  &lt;/p&gt;  &lt;p&gt;  &lt;font face="Arial" size="2"&gt;&lt;/font&gt;  &lt;/p&gt;  &lt;p&gt;  &lt;font face="Arial" size="2"&gt;PROD has been updated Successfully&lt;br&gt;&lt;a href=https://www.orange.com/en &gt; PROD Server &lt;/a&gt;&lt;/font&gt;  &lt;p&gt;  &lt;/p&gt;&lt;/br&gt;  &lt;font face="Arial" size="2"&gt;&lt;b&gt;Thanks and Regards&lt;/b&gt;  &lt;/font&gt;  &lt;/p&gt;  &lt;/body&gt;</t>
+  </si>
+  <si>
+    <t>XYZ1234@gmail.com</t>
+  </si>
+  <si>
+    <t>IJKL1234@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -520,7 +520,7 @@
         <v>9</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>6</v>
@@ -531,7 +531,7 @@
         <v>10</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C3" t="s">
         <v>6</v>
@@ -553,7 +553,7 @@
         <v>11</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C5" t="s">
         <v>6</v>
@@ -599,7 +599,7 @@
         <v>9</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>6</v>
@@ -610,7 +610,7 @@
         <v>10</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C3" t="s">
         <v>6</v>
@@ -632,7 +632,7 @@
         <v>11</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C5" t="s">
         <v>6</v>
@@ -640,10 +640,10 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1" xr:uid="{70BC05A0-A62A-44B0-999B-ACC357CEC35F}"/>
-    <hyperlink ref="B3" r:id="rId2" xr:uid="{9ED1D3CC-C3CD-45B8-B8C9-182F74F1E923}"/>
-    <hyperlink ref="B4" r:id="rId3" xr:uid="{590A581C-C901-43BB-9630-30EFFA676F77}"/>
-    <hyperlink ref="B5" r:id="rId4" xr:uid="{D642B6FB-8A7C-4024-A006-BA04376F12ED}"/>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{6435545F-5C33-41B0-8006-CC67232AAA23}"/>
+    <hyperlink ref="B3" r:id="rId2" xr:uid="{D7F58DC4-F2F7-4AB8-802E-DF2C9A55BE3F}"/>
+    <hyperlink ref="B4" r:id="rId3" xr:uid="{7ECB646F-1F72-462B-90CD-1D39FCD725A2}"/>
+    <hyperlink ref="B5" r:id="rId4" xr:uid="{7E1FB060-909A-4880-A779-8B50C8D9899C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -679,7 +679,7 @@
         <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>